<commit_message>
junit 5 and maven code
</commit_message>
<xml_diff>
--- a/src/test.demoApi/resources/testData/demoData.xlsx
+++ b/src/test.demoApi/resources/testData/demoData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fosman\IdeaProjects\mtf-dm-automation-test-api\src\test.demoApi\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3546B9-63D9-4988-8D7D-F48B3BF177C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F147D8CE-F00E-422B-A2CB-470B991622B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{3FAEF57A-74CB-4873-83C5-7175CED35448}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{3FAEF57A-74CB-4873-83C5-7175CED35448}"/>
   </bookViews>
   <sheets>
     <sheet name="Create" sheetId="1" r:id="rId1"/>
@@ -176,7 +176,7 @@
     <t>201</t>
   </si>
   <si>
-    <t>2024</t>
+    <t>2025</t>
   </si>
 </sst>
 </file>

</xml_diff>